<commit_message>
Agrega control contractual EPM, ajusta correos ANS y actualiza reglas de validación de materiales
</commit_message>
<xml_diff>
--- a/modules/informe_ans/config/SISTEMA_PARRILLA.xlsx
+++ b/modules/informe_ans/config/SISTEMA_PARRILLA.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hector.gaviria\Desktop\Launcher_Elite\modules\informe_ans\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1BEA14A8-193C-47FE-9ECC-0144DC2B611B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99A18238-3CC8-4C60-92F7-37BE29894ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{3FD0281D-E015-4104-BD1A-E246729E212C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="3">
   <si>
     <t>PEDIDO</t>
   </si>
@@ -54,13 +54,26 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -71,9 +84,18 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
       <right/>
       <top/>
       <bottom/>
@@ -83,16 +105,40 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -110,8 +156,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4302AFFF-EC3B-4DD7-848E-F59A29D4050F}" name="Tabla1" displayName="Tabla1" ref="A1:B3" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:B3" xr:uid="{4302AFFF-EC3B-4DD7-848E-F59A29D4050F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4302AFFF-EC3B-4DD7-848E-F59A29D4050F}" name="Tabla1" displayName="Tabla1" ref="A1:B17" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:B17" xr:uid="{4302AFFF-EC3B-4DD7-848E-F59A29D4050F}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{A0F9653D-9E42-4813-A4DF-8BD8F47ABB7C}" name="PEDIDO"/>
     <tableColumn id="2" xr3:uid="{5F8222D3-253E-4C3B-8778-0533702AE635}" name="OBSERVACION"/>
@@ -437,7 +483,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3ED12F5-5F90-49F6-AB60-93215FCDD301}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
@@ -467,10 +513,126 @@
         <v>2</v>
       </c>
     </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>23831988</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>23833690</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>23841064</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>23845645</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>23852770</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>23852783</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>23857705</v>
+      </c>
+      <c r="B10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
+        <v>23860597</v>
+      </c>
+      <c r="B11" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>23860687</v>
+      </c>
+      <c r="B12" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <v>23861942</v>
+      </c>
+      <c r="B13" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>23863446</v>
+      </c>
+      <c r="B14" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <v>23864911</v>
+      </c>
+      <c r="B15" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>23799664</v>
+      </c>
+      <c r="B16" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>23867551</v>
+      </c>
+      <c r="B17" t="s">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>